<commit_message>
feat: add Expected Annual Damage (EAD) analysis to Risk Dashboard
Implement trapezoidal integration across 7 return periods (2.3yr–500yr)
for all 42 flood scenarios, producing EAD values per climate, maintenance
level, district, and asset type (Agriculture, Kacha, Pakka, High-Rise).

- Add calculateEad() pure utility function in risk.ts
- Add useEadData hook computing all 240 EAD values
- Add EadBarChart component (Agriculture + Buildings stacked bar)
- Add RiskEadView with summary table, district chart, ranked table,
  and choropleth map integration (active by default)
- Wire EAD as 4th tab in RiskDashboard
- Update README, CHANGELOG, and CLAUDE.md
</commit_message>
<xml_diff>
--- a/Exposure_Stats/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
+++ b/Exposure_Stats/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TOTAL_Exp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TOTAL_Vul" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TOTAL_Dmg" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dadu_Exp" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Dadu_Vul" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Dadu_Dmg" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Jacobabad_Exp" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Jacobabad_Vul" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Jacobabad_Dmg" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Jamshoro_Exp" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Jamshoro_Vul" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Jamshoro_Dmg" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Larkana_Exp" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Larkana_Vul" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Larkana_Dmg" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Kashmore_Exp" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Kashmore_Vul" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Kashmore_Dmg" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Naushahro Feroze_Exp" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Naushahro Feroze_Vul" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Naushahro Feroze_Dmg" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Qambar Shahdadkot_Exp" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Qambar Shahdadkot_Vul" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Qambar Shahdadkot_Dmg" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Shaheed Benazirabad_Exp" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Shaheed Benazirabad_Vul" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Shaheed Benazirabad_Dmg" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Shikarpur_Exp" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Shikarpur_Vul" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Shikarpur_Dmg" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTAL_Exp" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTAL_Vul" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTAL_Dmg" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dadu_Exp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dadu_Vul" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dadu_Dmg" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jacobabad_Exp" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jacobabad_Vul" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jacobabad_Dmg" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jamshoro_Exp" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jamshoro_Vul" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jamshoro_Dmg" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Larkana_Exp" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Larkana_Vul" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Larkana_Dmg" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kashmore_Exp" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kashmore_Vul" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kashmore_Dmg" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Naushahro Feroze_Exp" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Naushahro Feroze_Vul" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Naushahro Feroze_Dmg" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Qambar Shahdadkot_Exp" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Qambar Shahdadkot_Vul" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Qambar Shahdadkot_Dmg" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shaheed Benazirabad_Exp" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shaheed Benazirabad_Vul" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shaheed Benazirabad_Dmg" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shikarpur_Exp" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shikarpur_Vul" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shikarpur_Dmg" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,17 +469,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -897,17 +897,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -1325,17 +1325,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -1748,22 +1748,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -2181,17 +2181,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -2609,17 +2609,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -3032,22 +3032,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -3465,17 +3465,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -3893,17 +3893,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -4316,22 +4316,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -4749,17 +4749,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -5177,17 +5177,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -5605,17 +5605,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -6028,22 +6028,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -6461,17 +6461,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -6889,17 +6889,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -7312,22 +7312,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -7745,17 +7745,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -8173,17 +8173,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -8596,22 +8596,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -9029,17 +9029,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -9457,17 +9457,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -9880,22 +9880,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -10308,22 +10308,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -10741,17 +10741,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -11169,17 +11169,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -11592,22 +11592,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>
@@ -12025,17 +12025,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -12453,17 +12453,17 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha (sqm)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka (sqm)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise (sqm)</t>
         </is>
       </c>
     </row>
@@ -12876,22 +12876,22 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Crop (ha)</t>
+          <t>Crop ($)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 56% (sqm)</t>
+          <t>Kacha ($)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Build &lt;3m 44% (sqm)</t>
+          <t>Pakka ($)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Build &gt;=3m (sqm)</t>
+          <t>High-rise ($)</t>
         </is>
       </c>
     </row>

</xml_diff>